<commit_message>
Inserido Coluna de auditor na planilha de resultados e implementado cálculo de nota da auditoria
</commit_message>
<xml_diff>
--- a/resultado_auditorias.xlsx
+++ b/resultado_auditorias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,27 +424,37 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Identificação do Auditor</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Ruim</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Regular</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Bom</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Ótimo</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>NA</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Nota (%)</t>
         </is>
       </c>
     </row>
@@ -454,20 +464,28 @@
           <t>CS1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>4</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ingrid Ferreira</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
         <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>55.68</v>
       </c>
     </row>
     <row r="3">
@@ -476,20 +494,28 @@
           <t>Portaria</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bruno Godoy</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>3</v>
       </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
       <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
         <v>10</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>3</v>
       </c>
-      <c r="F3" t="n">
-        <v>2</v>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>66.25</v>
       </c>
     </row>
     <row r="4">
@@ -498,20 +524,28 @@
           <t>CS1</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RODRIGO AZEVEDO </t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>5</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>14</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
       <c r="F4" t="n">
         <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>47.73</v>
       </c>
     </row>
     <row r="5">
@@ -520,20 +554,28 @@
           <t>CS2</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lucas Oliveira </t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
         <v>18</v>
       </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
       <c r="F5" t="n">
         <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>70.45</v>
       </c>
     </row>
     <row r="6">
@@ -542,20 +584,28 @@
           <t xml:space="preserve">Almox. Componente </t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>1</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fábio Oliveira </t>
+        </is>
       </c>
       <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
         <v>8</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>13</v>
       </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
       <c r="F6" t="n">
         <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>63.64</v>
       </c>
     </row>
     <row r="7">
@@ -564,20 +614,28 @@
           <t xml:space="preserve">Oficina - Ferramentaria </t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>0</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anderson Santos </t>
+        </is>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>16</v>
       </c>
-      <c r="E7" t="n">
-        <v>4</v>
-      </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -586,20 +644,28 @@
           <t xml:space="preserve">RH </t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>0</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fábio Oliveira </t>
+        </is>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>6</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>10</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>90.62</v>
       </c>
     </row>
     <row r="9">
@@ -608,20 +674,28 @@
           <t xml:space="preserve">Área da engenharia </t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>2</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gleidson Cunha </t>
+        </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>3</v>
       </c>
-      <c r="E9" t="n">
-        <v>4</v>
-      </c>
       <c r="F9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" t="n">
         <v>13</v>
+      </c>
+      <c r="H9" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="10">
@@ -630,20 +704,28 @@
           <t xml:space="preserve">Área recreativa </t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>2</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gleidson Cunha </t>
+        </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
         <v>2</v>
       </c>
       <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
         <v>12</v>
+      </c>
+      <c r="H10" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="11">
@@ -652,20 +734,28 @@
           <t xml:space="preserve">Plasma </t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>2</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ingrid Ferreira</t>
+        </is>
       </c>
       <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
         <v>17</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>3</v>
       </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
       <c r="F11" t="n">
         <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>51.14</v>
       </c>
     </row>
     <row r="12">
@@ -674,20 +764,28 @@
           <t>Teste</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>2</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingrid Ferreira </t>
+        </is>
       </c>
       <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
         <v>9</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>10</v>
       </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>59.52</v>
       </c>
     </row>
     <row r="13">
@@ -696,20 +794,28 @@
           <t>Teste</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>4</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingrid Ferreira </t>
+        </is>
       </c>
       <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="n">
         <v>7</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>11</v>
       </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
       <c r="F13" t="n">
         <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>57.95</v>
       </c>
     </row>
     <row r="14">
@@ -718,20 +824,28 @@
           <t>Teste</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>0</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingrid Ferreira </t>
+        </is>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
         <v>22</v>
       </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
       <c r="F14" t="n">
         <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="15">
@@ -740,20 +854,28 @@
           <t>Teste</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>0</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingrid Ferreira </t>
+        </is>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
         <v>22</v>
       </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
       <c r="F15" t="n">
         <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="16">
@@ -762,20 +884,28 @@
           <t>Engenharia</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>1</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Alexandre Evangelista</t>
+        </is>
       </c>
       <c r="C16" t="n">
         <v>1</v>
       </c>
       <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
         <v>15</v>
       </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
       <c r="F16" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" t="n">
+        <v>72.22</v>
       </c>
     </row>
     <row r="17">
@@ -784,20 +914,28 @@
           <t>Ferramantaria</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Anderson Silva Melo</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>13</v>
       </c>
-      <c r="C17" t="n">
-        <v>2</v>
-      </c>
       <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="n">
         <v>6</v>
       </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>41.67</v>
       </c>
     </row>
     <row r="18">
@@ -806,20 +944,28 @@
           <t>WP Solda</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emerson Paschoalino </t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>14</v>
       </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
       <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
         <v>3</v>
       </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
       <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
         <v>5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>33.82</v>
       </c>
     </row>
     <row r="19">
@@ -828,20 +974,28 @@
           <t xml:space="preserve">Expedição </t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kleber Geovan da Silva Borges </t>
+        </is>
+      </c>
+      <c r="C19" t="n">
         <v>3</v>
       </c>
-      <c r="C19" t="n">
-        <v>2</v>
-      </c>
       <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="n">
         <v>15</v>
       </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="20">
@@ -850,20 +1004,28 @@
           <t xml:space="preserve">Laser </t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>0</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marcelo Batista </t>
+        </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="n">
         <v>19</v>
       </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>72.62</v>
       </c>
     </row>
     <row r="21">
@@ -872,20 +1034,28 @@
           <t>Estoque wip</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>0</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lucas Acacio </t>
+        </is>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
         <v>15</v>
       </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
       <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
         <v>7</v>
+      </c>
+      <c r="H21" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="22">
@@ -894,20 +1064,28 @@
           <t>Escritório RH</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>0</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Jonathas</t>
+        </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
         <v>11</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>8</v>
+      </c>
+      <c r="H22" t="n">
+        <v>92.86</v>
       </c>
     </row>
     <row r="23">
@@ -916,20 +1094,28 @@
           <t>Usinagem chassis</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rodrigo Brito </t>
+        </is>
+      </c>
+      <c r="C23" t="n">
         <v>10</v>
       </c>
-      <c r="C23" t="n">
+      <c r="D23" t="n">
         <v>7</v>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>5</v>
       </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
       <c r="F23" t="n">
         <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>44.32</v>
       </c>
     </row>
     <row r="24">
@@ -938,20 +1124,28 @@
           <t>Escritório Qualidade</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>1</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sergio de Carvalho </t>
+        </is>
       </c>
       <c r="C24" t="n">
         <v>1</v>
       </c>
       <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
         <v>6</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>8</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>6</v>
+      </c>
+      <c r="H24" t="n">
+        <v>82.81</v>
       </c>
     </row>
     <row r="25">
@@ -960,20 +1154,28 @@
           <t xml:space="preserve">Solda/Dispositivos </t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sergio de Carvalho </t>
+        </is>
+      </c>
+      <c r="C25" t="n">
         <v>11</v>
       </c>
-      <c r="C25" t="n">
-        <v>4</v>
-      </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
         <v>5</v>
+      </c>
+      <c r="H25" t="n">
+        <v>36.76</v>
       </c>
     </row>
     <row r="26">
@@ -982,20 +1184,28 @@
           <t xml:space="preserve">Refeitório </t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>0</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kleber Geovan da Silva Borges </t>
+        </is>
       </c>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
         <v>19</v>
       </c>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>76.25</v>
       </c>
     </row>
     <row r="27">
@@ -1004,20 +1214,28 @@
           <t>Solda chassis</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>0</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ricardo de Oliveira </t>
+        </is>
       </c>
       <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
         <v>6</v>
       </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
         <v>16</v>
       </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
       <c r="F27" t="n">
         <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>68.18000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1026,20 +1244,28 @@
           <t xml:space="preserve">Célula de solda 4 - Banjos Scania </t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gleidson Pereira Cunha </t>
+        </is>
+      </c>
+      <c r="C28" t="n">
         <v>3</v>
       </c>
-      <c r="C28" t="n">
-        <v>2</v>
-      </c>
       <c r="D28" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E28" t="n">
         <v>8</v>
       </c>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="29">
@@ -1048,20 +1274,28 @@
           <t>Linha de banjo</t>
         </is>
       </c>
-      <c r="B29" t="n">
-        <v>4</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ricardo de Oliveira Santana </t>
+        </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
         <v>17</v>
       </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
       <c r="F29" t="n">
         <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>64.77</v>
       </c>
     </row>
     <row r="30">
@@ -1070,20 +1304,28 @@
           <t xml:space="preserve">Recebimento área externa </t>
         </is>
       </c>
-      <c r="B30" t="n">
-        <v>1</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job fialho </t>
+        </is>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
         <v>3</v>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>12</v>
       </c>
-      <c r="F30" t="n">
+      <c r="G30" t="n">
         <v>6</v>
+      </c>
+      <c r="H30" t="n">
+        <v>90.62</v>
       </c>
     </row>
     <row r="31">
@@ -1092,20 +1334,28 @@
           <t>Recebimento e qualidade</t>
         </is>
       </c>
-      <c r="B31" t="n">
-        <v>2</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>LUCIANO</t>
+        </is>
       </c>
       <c r="C31" t="n">
         <v>2</v>
       </c>
       <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
         <v>15</v>
       </c>
-      <c r="E31" t="n">
-        <v>2</v>
-      </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="n">
+        <v>70.23999999999999</v>
       </c>
     </row>
     <row r="32">
@@ -1114,20 +1364,28 @@
           <t xml:space="preserve">Escritório Manutenção </t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>2</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marcelo Sousa </t>
+        </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
         <v>10</v>
       </c>
-      <c r="E32" t="n">
+      <c r="F32" t="n">
         <v>3</v>
       </c>
-      <c r="F32" t="n">
+      <c r="G32" t="n">
         <v>6</v>
+      </c>
+      <c r="H32" t="n">
+        <v>71.88</v>
       </c>
     </row>
     <row r="33">
@@ -1136,20 +1394,28 @@
           <t>RESERVATORIO</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>4</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MARCELO SOUSA</t>
+        </is>
       </c>
       <c r="C33" t="n">
         <v>4</v>
       </c>
       <c r="D33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" t="n">
         <v>10</v>
       </c>
-      <c r="E33" t="n">
-        <v>4</v>
-      </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>65.91</v>
       </c>
     </row>
     <row r="34">
@@ -1158,20 +1424,28 @@
           <t>Almoxarifado Componentes</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Breno Lamac </t>
+        </is>
+      </c>
+      <c r="C34" t="n">
         <v>9</v>
       </c>
-      <c r="C34" t="n">
-        <v>4</v>
-      </c>
       <c r="D34" t="n">
+        <v>4</v>
+      </c>
+      <c r="E34" t="n">
         <v>8</v>
       </c>
-      <c r="E34" t="n">
-        <v>0</v>
-      </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="n">
+        <v>48.81</v>
       </c>
     </row>
     <row r="35">
@@ -1180,20 +1454,28 @@
           <t xml:space="preserve">Pátio Externo </t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Fabio dos Anjos Paes</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
         <v>6</v>
       </c>
-      <c r="C35" t="n">
-        <v>4</v>
-      </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
         <v>12</v>
+      </c>
+      <c r="H35" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="36">
@@ -1202,20 +1484,28 @@
           <t>Estanqueidade care</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>1</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Humberto Victor </t>
+        </is>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" t="n">
         <v>18</v>
       </c>
-      <c r="E36" t="n">
-        <v>0</v>
-      </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" t="n">
+        <v>70.23999999999999</v>
       </c>
     </row>
     <row r="37">
@@ -1224,20 +1514,28 @@
           <t xml:space="preserve">Estoque de componentes. </t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>0</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lucas Oliveira </t>
+        </is>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="n">
         <v>15</v>
       </c>
-      <c r="E37" t="n">
-        <v>0</v>
-      </c>
       <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
         <v>5</v>
+      </c>
+      <c r="H37" t="n">
+        <v>72.06</v>
       </c>
     </row>
     <row r="38">
@@ -1246,20 +1544,28 @@
           <t xml:space="preserve">Escritório ferramentaria </t>
         </is>
       </c>
-      <c r="B38" t="n">
-        <v>0</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lucas Oliveira </t>
+        </is>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D38" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" t="n">
         <v>16</v>
       </c>
-      <c r="E38" t="n">
-        <v>0</v>
-      </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="39">
@@ -1268,20 +1574,28 @@
           <t>Portaria RH</t>
         </is>
       </c>
-      <c r="B39" t="n">
-        <v>2</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marlon de Paula. </t>
+        </is>
       </c>
       <c r="C39" t="n">
         <v>2</v>
       </c>
       <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="n">
         <v>5</v>
       </c>
-      <c r="E39" t="n">
+      <c r="F39" t="n">
         <v>9</v>
       </c>
-      <c r="F39" t="n">
-        <v>4</v>
+      <c r="G39" t="n">
+        <v>4</v>
+      </c>
+      <c r="H39" t="n">
+        <v>79.17</v>
       </c>
     </row>
     <row r="40">
@@ -1290,20 +1604,28 @@
           <t>Oficina - Ferramentaria</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>2</v>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alexandre Evangelista </t>
+        </is>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D40" t="n">
+        <v>4</v>
+      </c>
+      <c r="E40" t="n">
         <v>12</v>
       </c>
-      <c r="E40" t="n">
-        <v>0</v>
-      </c>
       <c r="F40" t="n">
-        <v>4</v>
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>4</v>
+      </c>
+      <c r="H40" t="n">
+        <v>63.89</v>
       </c>
     </row>
     <row r="41">
@@ -1312,20 +1634,28 @@
           <t xml:space="preserve">Escritório da logística </t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>1</v>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gleidson Cunha </t>
+        </is>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
         <v>8</v>
       </c>
-      <c r="E41" t="n">
+      <c r="F41" t="n">
         <v>6</v>
       </c>
-      <c r="F41" t="n">
+      <c r="G41" t="n">
         <v>7</v>
+      </c>
+      <c r="H41" t="n">
+        <v>81.67</v>
       </c>
     </row>
     <row r="42">
@@ -1334,20 +1664,28 @@
           <t xml:space="preserve">Área Recreativa </t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>4</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Marcelo. B</t>
+        </is>
       </c>
       <c r="C42" t="n">
+        <v>4</v>
+      </c>
+      <c r="D42" t="n">
         <v>6</v>
       </c>
-      <c r="D42" t="n">
+      <c r="E42" t="n">
         <v>8</v>
       </c>
-      <c r="E42" t="n">
-        <v>0</v>
-      </c>
       <c r="F42" t="n">
-        <v>4</v>
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>4</v>
+      </c>
+      <c r="H42" t="n">
+        <v>55.56</v>
       </c>
     </row>
     <row r="43">
@@ -1356,20 +1694,28 @@
           <t>Protótipos</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Breno Lamac</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
         <v>6</v>
-      </c>
-      <c r="C43" t="n">
-        <v>5</v>
       </c>
       <c r="D43" t="n">
         <v>5</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
         <v>6</v>
+      </c>
+      <c r="H43" t="n">
+        <v>48.44</v>
       </c>
     </row>
     <row r="44">
@@ -1378,20 +1724,28 @@
           <t xml:space="preserve">Pintura </t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marcelo Sousa </t>
+        </is>
+      </c>
+      <c r="C44" t="n">
         <v>3</v>
       </c>
-      <c r="C44" t="n">
-        <v>2</v>
-      </c>
       <c r="D44" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" t="n">
         <v>13</v>
       </c>
-      <c r="E44" t="n">
-        <v>4</v>
-      </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>70.45</v>
       </c>
     </row>
     <row r="45">
@@ -1400,20 +1754,28 @@
           <t xml:space="preserve">Escritório engenharia </t>
         </is>
       </c>
-      <c r="B45" t="n">
-        <v>0</v>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jonathas Andrade </t>
+        </is>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D45" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" t="n">
         <v>8</v>
       </c>
-      <c r="E45" t="n">
-        <v>4</v>
-      </c>
       <c r="F45" t="n">
+        <v>4</v>
+      </c>
+      <c r="G45" t="n">
         <v>8</v>
+      </c>
+      <c r="H45" t="n">
+        <v>78.56999999999999</v>
       </c>
     </row>
     <row r="46">
@@ -1422,20 +1784,28 @@
           <t>Portaria</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Alexandre Evangelista</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
         <v>8</v>
       </c>
-      <c r="C46" t="n">
-        <v>0</v>
-      </c>
       <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
         <v>10</v>
       </c>
-      <c r="E46" t="n">
-        <v>0</v>
-      </c>
       <c r="F46" t="n">
-        <v>4</v>
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>4</v>
+      </c>
+      <c r="H46" t="n">
+        <v>52.78</v>
       </c>
     </row>
     <row r="47">
@@ -1444,20 +1814,28 @@
           <t>Usinagem de eixos</t>
         </is>
       </c>
-      <c r="B47" t="n">
-        <v>2</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Humberto </t>
+        </is>
       </c>
       <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
         <v>3</v>
       </c>
-      <c r="D47" t="n">
+      <c r="E47" t="n">
         <v>16</v>
       </c>
-      <c r="E47" t="n">
-        <v>0</v>
-      </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" t="n">
+        <v>66.67</v>
       </c>
     </row>
     <row r="48">
@@ -1466,20 +1844,28 @@
           <t>Robô nba</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>4</v>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kleber Geovan da Silva Borges </t>
+        </is>
       </c>
       <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="n">
         <v>7</v>
       </c>
-      <c r="D48" t="n">
+      <c r="E48" t="n">
         <v>5</v>
       </c>
-      <c r="E48" t="n">
-        <v>2</v>
-      </c>
       <c r="F48" t="n">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="G48" t="n">
+        <v>4</v>
+      </c>
+      <c r="H48" t="n">
+        <v>56.94</v>
       </c>
     </row>
     <row r="49">
@@ -1488,20 +1874,28 @@
           <t>ETE</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bruno Godoy</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
         <v>11</v>
       </c>
-      <c r="C49" t="n">
-        <v>1</v>
-      </c>
       <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
         <v>6</v>
       </c>
-      <c r="E49" t="n">
-        <v>1</v>
-      </c>
       <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="n">
         <v>3</v>
+      </c>
+      <c r="H49" t="n">
+        <v>46.05</v>
       </c>
     </row>
     <row r="50">
@@ -1510,20 +1904,28 @@
           <t>RH</t>
         </is>
       </c>
-      <c r="B50" t="n">
-        <v>0</v>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Anderson Melo</t>
+        </is>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D50" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" t="n">
         <v>11</v>
       </c>
-      <c r="E50" t="n">
+      <c r="F50" t="n">
         <v>8</v>
       </c>
-      <c r="F50" t="n">
-        <v>1</v>
+      <c r="G50" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" t="n">
+        <v>82.14</v>
       </c>
     </row>
     <row r="51">
@@ -1532,20 +1934,28 @@
           <t xml:space="preserve">Estoque de WP Estamparia </t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emerson Paschoalino </t>
+        </is>
+      </c>
+      <c r="C51" t="n">
         <v>11</v>
       </c>
-      <c r="C51" t="n">
+      <c r="D51" t="n">
         <v>5</v>
       </c>
-      <c r="D51" t="n">
-        <v>4</v>
-      </c>
       <c r="E51" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F51" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" t="n">
+        <v>41.25</v>
       </c>
     </row>
     <row r="52">
@@ -1554,20 +1964,28 @@
           <t xml:space="preserve">Metrologia </t>
         </is>
       </c>
-      <c r="B52" t="n">
-        <v>1</v>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marcelo Sousa </t>
+        </is>
       </c>
       <c r="C52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
         <v>16</v>
       </c>
-      <c r="E52" t="n">
-        <v>1</v>
-      </c>
       <c r="F52" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="G52" t="n">
+        <v>4</v>
+      </c>
+      <c r="H52" t="n">
+        <v>73.61</v>
       </c>
     </row>
     <row r="53">
@@ -1576,20 +1994,28 @@
           <t>Laser</t>
         </is>
       </c>
-      <c r="B53" t="n">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Anderson Silva Melo</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
         <v>13</v>
       </c>
-      <c r="C53" t="n">
+      <c r="D53" t="n">
         <v>5</v>
       </c>
-      <c r="D53" t="n">
+      <c r="E53" t="n">
         <v>3</v>
       </c>
-      <c r="E53" t="n">
-        <v>0</v>
-      </c>
       <c r="F53" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="n">
+        <v>38.1</v>
       </c>
     </row>
     <row r="54">
@@ -1598,20 +2024,28 @@
           <t>Estoque do WIP solda</t>
         </is>
       </c>
-      <c r="B54" t="n">
-        <v>5</v>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Alan Gomes</t>
+        </is>
       </c>
       <c r="C54" t="n">
         <v>5</v>
       </c>
       <c r="D54" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E54" t="n">
+        <v>4</v>
+      </c>
+      <c r="F54" t="n">
         <v>3</v>
       </c>
-      <c r="F54" t="n">
+      <c r="G54" t="n">
         <v>5</v>
+      </c>
+      <c r="H54" t="n">
+        <v>57.35</v>
       </c>
     </row>
     <row r="55">
@@ -1620,20 +2054,28 @@
           <t>Estoque de Matéria Prima</t>
         </is>
       </c>
-      <c r="B55" t="n">
-        <v>5</v>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Breno Lamac</t>
+        </is>
       </c>
       <c r="C55" t="n">
         <v>5</v>
       </c>
       <c r="D55" t="n">
+        <v>5</v>
+      </c>
+      <c r="E55" t="n">
         <v>7</v>
       </c>
-      <c r="E55" t="n">
-        <v>0</v>
-      </c>
       <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
         <v>5</v>
+      </c>
+      <c r="H55" t="n">
+        <v>52.94</v>
       </c>
     </row>
     <row r="56">
@@ -1642,20 +2084,28 @@
           <t xml:space="preserve">Dobradeiras </t>
         </is>
       </c>
-      <c r="B56" t="n">
-        <v>2</v>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marcelo Sousa </t>
+        </is>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="n">
         <v>18</v>
       </c>
-      <c r="E56" t="n">
-        <v>0</v>
-      </c>
       <c r="F56" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G56" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" t="n">
+        <v>69.05</v>
       </c>
     </row>
     <row r="57">
@@ -1664,20 +2114,28 @@
           <t>Almoxarifado de componentes</t>
         </is>
       </c>
-      <c r="B57" t="n">
-        <v>4</v>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alan Gomes </t>
+        </is>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="n">
         <v>5</v>
       </c>
-      <c r="E57" t="n">
+      <c r="F57" t="n">
         <v>10</v>
       </c>
-      <c r="F57" t="n">
+      <c r="G57" t="n">
         <v>3</v>
+      </c>
+      <c r="H57" t="n">
+        <v>77.63</v>
       </c>
     </row>
     <row r="58">
@@ -1686,20 +2144,28 @@
           <t>Reservatorio</t>
         </is>
       </c>
-      <c r="B58" t="n">
-        <v>1</v>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Eduardo Fialho </t>
+        </is>
       </c>
       <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
         <v>3</v>
       </c>
-      <c r="D58" t="n">
+      <c r="E58" t="n">
         <v>18</v>
       </c>
-      <c r="E58" t="n">
-        <v>0</v>
-      </c>
       <c r="F58" t="n">
         <v>0</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>69.31999999999999</v>
       </c>
     </row>
     <row r="59">
@@ -1708,20 +2174,28 @@
           <t xml:space="preserve">Oficina de manutenção </t>
         </is>
       </c>
-      <c r="B59" t="n">
-        <v>2</v>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUCIANO NASCIMENTO </t>
+        </is>
       </c>
       <c r="C59" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D59" t="n">
+        <v>4</v>
+      </c>
+      <c r="E59" t="n">
         <v>14</v>
       </c>
-      <c r="E59" t="n">
-        <v>2</v>
-      </c>
       <c r="F59" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>68.18000000000001</v>
       </c>
     </row>
     <row r="60">
@@ -1730,20 +2204,28 @@
           <t xml:space="preserve">Recebimento-Logística </t>
         </is>
       </c>
-      <c r="B60" t="n">
-        <v>1</v>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sergio de Carvalho </t>
+        </is>
       </c>
       <c r="C60" t="n">
         <v>1</v>
       </c>
       <c r="D60" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" t="n">
         <v>10</v>
       </c>
-      <c r="E60" t="n">
+      <c r="F60" t="n">
         <v>6</v>
       </c>
-      <c r="F60" t="n">
-        <v>4</v>
+      <c r="G60" t="n">
+        <v>4</v>
+      </c>
+      <c r="H60" t="n">
+        <v>79.17</v>
       </c>
     </row>
     <row r="61">
@@ -1752,20 +2234,28 @@
           <t>Pintura</t>
         </is>
       </c>
-      <c r="B61" t="n">
-        <v>7</v>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Ricardo Santana</t>
+        </is>
       </c>
       <c r="C61" t="n">
         <v>7</v>
       </c>
       <c r="D61" t="n">
+        <v>7</v>
+      </c>
+      <c r="E61" t="n">
         <v>8</v>
       </c>
-      <c r="E61" t="n">
-        <v>0</v>
-      </c>
       <c r="F61" t="n">
         <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="n">
+        <v>51.14</v>
       </c>
     </row>
     <row r="62">
@@ -1774,20 +2264,28 @@
           <t xml:space="preserve">Dobradeira </t>
         </is>
       </c>
-      <c r="B62" t="n">
-        <v>2</v>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Humberto Victor </t>
+        </is>
       </c>
       <c r="C62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" t="n">
         <v>5</v>
       </c>
-      <c r="D62" t="n">
+      <c r="E62" t="n">
         <v>10</v>
       </c>
-      <c r="E62" t="n">
-        <v>2</v>
-      </c>
       <c r="F62" t="n">
+        <v>2</v>
+      </c>
+      <c r="G62" t="n">
         <v>3</v>
+      </c>
+      <c r="H62" t="n">
+        <v>65.79000000000001</v>
       </c>
     </row>
     <row r="63">
@@ -1796,20 +2294,28 @@
           <t xml:space="preserve">Logística/Expedição </t>
         </is>
       </c>
-      <c r="B63" t="n">
-        <v>0</v>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anderson Santos </t>
+        </is>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D63" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E63" t="n">
         <v>10</v>
       </c>
       <c r="F63" t="n">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="G63" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" t="n">
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="64">
@@ -1818,20 +2324,28 @@
           <t xml:space="preserve">SOLDA CHASSIS </t>
         </is>
       </c>
-      <c r="B64" t="n">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emerson Paschoalino </t>
+        </is>
+      </c>
+      <c r="C64" t="n">
         <v>13</v>
       </c>
-      <c r="C64" t="n">
-        <v>2</v>
-      </c>
       <c r="D64" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" t="n">
         <v>7</v>
       </c>
-      <c r="E64" t="n">
-        <v>0</v>
-      </c>
       <c r="F64" t="n">
         <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="n">
+        <v>43.18</v>
       </c>
     </row>
     <row r="65">
@@ -1840,20 +2354,28 @@
           <t>Sala ferramentaria</t>
         </is>
       </c>
-      <c r="B65" t="n">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Alexandre Evangelista</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
         <v>5</v>
       </c>
-      <c r="C65" t="n">
-        <v>0</v>
-      </c>
       <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
         <v>16</v>
       </c>
-      <c r="E65" t="n">
-        <v>0</v>
-      </c>
       <c r="F65" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" t="n">
+        <v>63.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>